<commit_message>
Update CPIExcel.xlsx with new package entry
</commit_message>
<xml_diff>
--- a/CPIExcel.xlsx
+++ b/CPIExcel.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="26">
   <si>
     <t>Package Name</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>ValueMapping</t>
+  </si>
+  <si>
+    <t>AnkushTesting</t>
+  </si>
+  <si>
+    <t>IDOC_-_SFTP_ASYN_AKD</t>
+  </si>
+  <si>
+    <t>1.0.11</t>
+  </si>
+  <si>
+    <t>2026-03-01</t>
   </si>
 </sst>
 </file>
@@ -481,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D912091-F28B-419E-969A-749E76A8C8AF}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="25.26953125"/>
@@ -707,6 +719,26 @@
         <v>18</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>